<commit_message>
Baza adresow klubow: kluby z listy kontaktow i puste wiersze
- 24 wiersze „Do uzupelnienia” (I liga i akademie CLJ U15) dostaly adres
  obiektu, e-mail, zrodlo i status.
- 35 nowych klubow z listy kontaktow (Liga / grupa = „Kontakty (spoza bazy)”).
- Uwagi przy KS CK Troszyn (e-mail z FB klubu, kontakt „KSC Krotoszyn”),
  Mlawiance Mlawa (kontakt „MKS Mlawa”) i SSM Wisla Plock.
- Test: kazdy klub ma juz adres albo e-mail, wiec sprawdzamy kluby bez adresu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RAbyht9gQjutBV1ng5Ztzu
</commit_message>
<xml_diff>
--- a/Kluby_Polska_Adresy.xlsx
+++ b/Kluby_Polska_Adresy.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Podsumowanie" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Adresy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adresy" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Adresy'!$A$1:$H$272</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Adresy'!$A$1:$H$307</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -488,6 +488,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -565,7 +566,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>nie sprawdzono – limit wyszukiwań w sesji</t>
+          <t>brak adresu – nie znaleziono w źródłach klubu/związku/gminy (szczegóły w Uwagach)</t>
         </is>
       </c>
     </row>
@@ -579,7 +580,6 @@
         <f>COUNTA(Adresy!B:B)-1</f>
         <v/>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -591,7 +591,6 @@
         <f>COUNTIF(Adresy!D:D,"?*")</f>
         <v/>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -603,8 +602,8 @@
         <f>COUNTIF(Adresy!E:E,"*@*")</f>
         <v/>
       </c>
-      <c r="C10" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -623,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H272"/>
+  <dimension ref="A1:H307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1144,7 +1143,11 @@
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>na liście kontaktów jako „MKS Mława” (ten sam e-mail mksmlawa@gmail.com)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1251,7 +1254,11 @@
           <t>Stadion gminny, 07-405 Troszyn</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr"/>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>kscktroszyn1@gmail.com</t>
+        </is>
+      </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
           <t>https://www.facebook.com/KSTROSZYN/</t>
@@ -1264,7 +1271,7 @@
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>ulicy i e-maila nie znalazłem; kontakt przez FB</t>
+          <t>ulicy i e-maila nie znalazłem; kontakt przez FB; e-mail kscktroszyn1@gmail.com z profilu klubu na FB; na liście kontaktów jako „KSC Krotoszyn” – to ten klub (nie Krotoszyn); boisko przy ul. Wesołej/Słowackiego – do potwierdzenia</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7953,7 @@
       </c>
       <c r="H187" s="8" t="inlineStr">
         <is>
-          <t>akademia – boisko treningowe i e-mail do uzupełnienia</t>
+          <t>akademia – boisko treningowe i e-mail do uzupełnienia; na liście kontaktów jako „Wisła Płock Akademia” (akademia.plock@gmail.com – nie znalazłem tego adresu w źródłach klubu); sekretariat klubu: poczta@wisla-plock.pl, tel. 24 367 65 20 (wisla-plock.pl/klub/kontakt/)</t>
         </is>
       </c>
     </row>
@@ -8004,17 +8011,29 @@
           <t>Niewiadów</t>
         </is>
       </c>
-      <c r="D189" s="8" t="inlineStr"/>
-      <c r="E189" s="8" t="inlineStr"/>
-      <c r="F189" s="8" t="inlineStr"/>
-      <c r="G189" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D189" s="8" t="inlineStr">
+        <is>
+          <t>Gminny Stadion Sportowy w Niewiadowie, Osiedle Niewiadów 40, 97-225 Ujazd</t>
+        </is>
+      </c>
+      <c r="E189" s="8" t="inlineStr">
+        <is>
+          <t>stal@stalniewiadow.pl</t>
+        </is>
+      </c>
+      <c r="F189" s="8" t="inlineStr">
+        <is>
+          <t>https://stalniewiadow.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G189" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H189" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>siedziba klubu: Osiedle Niewiadów 27; obiekt prowadzi MCS Ujazd</t>
         </is>
       </c>
     </row>
@@ -8072,17 +8091,29 @@
           <t>Białystok</t>
         </is>
       </c>
-      <c r="D191" s="8" t="inlineStr"/>
-      <c r="E191" s="8" t="inlineStr"/>
-      <c r="F191" s="8" t="inlineStr"/>
-      <c r="G191" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D191" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Kościelna 3, 15-087 Białystok</t>
+        </is>
+      </c>
+      <c r="E191" s="8" t="inlineStr">
+        <is>
+          <t>talent@aptalent.pl</t>
+        </is>
+      </c>
+      <c r="F191" s="8" t="inlineStr">
+        <is>
+          <t>https://www.aptalent.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G191" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H191" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>znaleziona tylko siedziba; akademia trenuje m.in. na kompleksie boisk Stadionu Miejskiego (ul. Słoneczna 1) – boisko meczowe U15 do potwierdzenia; tel. 690 913 999</t>
         </is>
       </c>
     </row>
@@ -8140,17 +8171,29 @@
           <t>Warszawa</t>
         </is>
       </c>
-      <c r="D193" s="8" t="inlineStr"/>
-      <c r="E193" s="8" t="inlineStr"/>
-      <c r="F193" s="8" t="inlineStr"/>
-      <c r="G193" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D193" s="8" t="inlineStr">
+        <is>
+          <t>Boisko Varsovii, ul. Międzyparkowa 4, 00-208 Warszawa</t>
+        </is>
+      </c>
+      <c r="E193" s="8" t="inlineStr">
+        <is>
+          <t>varsovia@varsovia.waw.pl</t>
+        </is>
+      </c>
+      <c r="F193" s="8" t="inlineStr">
+        <is>
+          <t>https://varsovia.waw.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G193" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H193" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>adres klubu; mecze grane też na obiekcie Hutnika (Aktywna Warszawa) i przy ul. Fleminga 2 – obiekt meczowy U15 do potwierdzenia; tel. 22 831 17 66</t>
         </is>
       </c>
     </row>
@@ -8204,17 +8247,29 @@
           <t>Szczecin</t>
         </is>
       </c>
-      <c r="D195" s="8" t="inlineStr"/>
-      <c r="E195" s="8" t="inlineStr"/>
-      <c r="F195" s="8" t="inlineStr"/>
-      <c r="G195" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D195" s="8" t="inlineStr">
+        <is>
+          <t>Football Park Szczecin, ul. Klonowica 3, 71-241 Szczecin</t>
+        </is>
+      </c>
+      <c r="E195" s="8" t="inlineStr">
+        <is>
+          <t>szczecin@footballacademy.pl</t>
+        </is>
+      </c>
+      <c r="F195" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fase.com.pl/infrastruktura/obiekty-treningowe</t>
+        </is>
+      </c>
+      <c r="G195" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H195" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>własne centrum piłkarskie FASE; korzysta też z Centrum Piłkarskiego MOSRiR (ul. Kresowa 42); sekretariat szkoły: sekretariat@fase.com.pl, tel. 735 631 783; e-mail biura FA Szczecin z footballacademy.pl</t>
         </is>
       </c>
     </row>
@@ -8386,17 +8441,29 @@
           <t>Poznań</t>
         </is>
       </c>
-      <c r="D200" s="8" t="inlineStr"/>
-      <c r="E200" s="8" t="inlineStr"/>
-      <c r="F200" s="8" t="inlineStr"/>
-      <c r="G200" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D200" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Warty „Ogródek”, ul. Droga Dębińska 12, 61-001 Poznań</t>
+        </is>
+      </c>
+      <c r="E200" s="8" t="inlineStr">
+        <is>
+          <t>akademia@wartapoznan.pl</t>
+        </is>
+      </c>
+      <c r="F200" s="8" t="inlineStr">
+        <is>
+          <t>https://wartapoznan.pl/</t>
+        </is>
+      </c>
+      <c r="G200" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H200" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>adres stadionu pierwszej drużyny – boisko meczowe U15 do potwierdzenia; ogólny e-mail klubu: info@wartapoznan.pl</t>
         </is>
       </c>
     </row>
@@ -8572,17 +8639,29 @@
           <t>Szczecin</t>
         </is>
       </c>
-      <c r="D205" s="8" t="inlineStr"/>
-      <c r="E205" s="8" t="inlineStr"/>
-      <c r="F205" s="8" t="inlineStr"/>
-      <c r="G205" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D205" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Witkiewicza 64, 71-215 Szczecin</t>
+        </is>
+      </c>
+      <c r="E205" s="8" t="inlineStr">
+        <is>
+          <t>salos@salesianum.pl</t>
+        </is>
+      </c>
+      <c r="F205" s="8" t="inlineStr">
+        <is>
+          <t>https://bip.um.szczecin.pl/files/7897A68FBB9E4E3C8746E2900D3A641C/153_md_2023_01_szkolenie_dziec.pdf</t>
+        </is>
+      </c>
+      <c r="G205" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H205" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>dane SL Salos z ofert w BIP UM Szczecin (2022–2023); boisko meczowe do potwierdzenia na salos.szczecin.pl; tel. 512 328 460</t>
         </is>
       </c>
     </row>
@@ -8602,17 +8681,29 @@
           <t>Poznań</t>
         </is>
       </c>
-      <c r="D206" s="8" t="inlineStr"/>
-      <c r="E206" s="8" t="inlineStr"/>
-      <c r="F206" s="8" t="inlineStr"/>
-      <c r="G206" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D206" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Źródlana 19/1, 60-642 Poznań</t>
+        </is>
+      </c>
+      <c r="E206" s="8" t="inlineStr">
+        <is>
+          <t>info@aprlampart.pl</t>
+        </is>
+      </c>
+      <c r="F206" s="8" t="inlineStr">
+        <is>
+          <t>https://www.poznan.pl/mim/main/kluby-i-stowarzyszenia-sportowe,poi,82/akademia-pilkarskiego-rozwoju-lampart,78290.html</t>
+        </is>
+      </c>
+      <c r="G206" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H206" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>do 06.2025 Akademia Piłkarska Reissa (na liście kontaktów jako „Akademia Reissa”, t.karkoszka@akademiareissa.pl); znaleziona tylko siedziba – boisko meczowe U15 do potwierdzenia; tel. 502 741 749; strona aprlampart.pl</t>
         </is>
       </c>
     </row>
@@ -8632,17 +8723,29 @@
           <t>Szczecin</t>
         </is>
       </c>
-      <c r="D207" s="8" t="inlineStr"/>
-      <c r="E207" s="8" t="inlineStr"/>
-      <c r="F207" s="8" t="inlineStr"/>
-      <c r="G207" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D207" s="8" t="inlineStr">
+        <is>
+          <t>Football Arena, al. Wojska Polskiego 246, 71-256 Szczecin</t>
+        </is>
+      </c>
+      <c r="E207" s="8" t="inlineStr">
+        <is>
+          <t>akademia@footballarena.pl</t>
+        </is>
+      </c>
+      <c r="F207" s="8" t="inlineStr">
+        <is>
+          <t>https://bip.um.szczecin.pl/files/B996EE3F2B5645208F970738893C89D0/430_md_2025_01_wsparcie_pilki_anon.pdf</t>
+        </is>
+      </c>
+      <c r="G207" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H207" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>dane Stowarzyszenia Football Arena z ofert w BIP UM Szczecin (2021–2025): 2 boiska pod balonem + 1 odkryte; tel. 696 046 000</t>
         </is>
       </c>
     </row>
@@ -8730,17 +8833,29 @@
           <t>Katowice</t>
         </is>
       </c>
-      <c r="D210" s="8" t="inlineStr"/>
-      <c r="E210" s="8" t="inlineStr"/>
-      <c r="F210" s="8" t="inlineStr"/>
-      <c r="G210" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D210" s="8" t="inlineStr">
+        <is>
+          <t>Akademia GKS Katowice, ul. Bukowa 1A, 40-108 Katowice</t>
+        </is>
+      </c>
+      <c r="E210" s="8" t="inlineStr">
+        <is>
+          <t>biuro@gkskatowice.eu</t>
+        </is>
+      </c>
+      <c r="F210" s="8" t="inlineStr">
+        <is>
+          <t>https://akademia.gkskatowice.eu/kontakt</t>
+        </is>
+      </c>
+      <c r="G210" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H210" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>adres akademii (siedziba) – boisko meczowe U15 do potwierdzenia; e-mail akademii zamaskowany na stronie, podany ogólny e-mail spółki (bip.gkskatowice.eu); tel. akademii 725 250 897</t>
         </is>
       </c>
     </row>
@@ -8760,17 +8875,29 @@
           <t>Wrocław</t>
         </is>
       </c>
-      <c r="D211" s="8" t="inlineStr"/>
-      <c r="E211" s="8" t="inlineStr"/>
-      <c r="F211" s="8" t="inlineStr"/>
-      <c r="G211" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D211" s="8" t="inlineStr">
+        <is>
+          <t>Kompleks Piłkarski „Oławka”, ul. Na Niskich Łąkach 8, Wrocław</t>
+        </is>
+      </c>
+      <c r="E211" s="8" t="inlineStr">
+        <is>
+          <t>b.mazur@fcwroclaw.pl</t>
+        </is>
+      </c>
+      <c r="F211" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcwroclaw.pl/obiekty/</t>
+        </is>
+      </c>
+      <c r="G211" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H211" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>trampkarze i juniorzy trenują na „Oławce” oraz na Polach Marsowych (al. Paderewskiego 35) – boisko meczowe U15 i kod pocztowy do potwierdzenia; biuro: ul. Kwidzyńska 33, 51-415 Wrocław, tel. 881 001 156; b.mazur = koordynator sportowy (rozgrywki); ogólnego e-maila brak</t>
         </is>
       </c>
     </row>
@@ -8984,17 +9111,29 @@
           <t>Opole</t>
         </is>
       </c>
-      <c r="D217" s="8" t="inlineStr"/>
-      <c r="E217" s="8" t="inlineStr"/>
-      <c r="F217" s="8" t="inlineStr"/>
-      <c r="G217" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D217" s="8" t="inlineStr">
+        <is>
+          <t>Itaka Arena (Stadion Miejski), ul. Leonarda Olejnika 1, 45-839 Opole</t>
+        </is>
+      </c>
+      <c r="E217" s="8" t="inlineStr">
+        <is>
+          <t>klub@odraopole.pl</t>
+        </is>
+      </c>
+      <c r="F217" s="8" t="inlineStr">
+        <is>
+          <t>https://odraopole.pl/en/kontakt</t>
+        </is>
+      </c>
+      <c r="G217" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H217" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>adres stadionu pierwszej drużyny – boisko meczowe U15 do potwierdzenia; e-mail ogólny klubu</t>
         </is>
       </c>
     </row>
@@ -9238,17 +9377,29 @@
           <t>Krosno</t>
         </is>
       </c>
-      <c r="D224" s="8" t="inlineStr"/>
-      <c r="E224" s="8" t="inlineStr"/>
-      <c r="F224" s="8" t="inlineStr"/>
-      <c r="G224" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D224" s="8" t="inlineStr">
+        <is>
+          <t>Profbud Arena, ul. Bohaterów Westerplatte 20, 38-400 Krosno</t>
+        </is>
+      </c>
+      <c r="E224" s="8" t="inlineStr">
+        <is>
+          <t>kontakt@beniaminek.org</t>
+        </is>
+      </c>
+      <c r="F224" s="8" t="inlineStr">
+        <is>
+          <t>https://beniaminek.org/kontakt/</t>
+        </is>
+      </c>
+      <c r="G224" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H224" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>pełnowymiarowe boisko ze sztuczną murawą; tel. 668 835 779; siedziba rejestrowa ul. Hallera 8/15</t>
         </is>
       </c>
     </row>
@@ -9306,17 +9457,29 @@
           <t>Kraków</t>
         </is>
       </c>
-      <c r="D226" s="8" t="inlineStr"/>
-      <c r="E226" s="8" t="inlineStr"/>
-      <c r="F226" s="8" t="inlineStr"/>
-      <c r="G226" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D226" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Garbarni, ul. Rydlówka 21G, 30-363 Kraków</t>
+        </is>
+      </c>
+      <c r="E226" s="8" t="inlineStr">
+        <is>
+          <t>sekretariat@garbarnia.krakow.pl</t>
+        </is>
+      </c>
+      <c r="F226" s="8" t="inlineStr">
+        <is>
+          <t>https://garbarnia.krakow.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G226" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H226" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>akademia: akademia@garbarnia.krakow.pl, tel. 736 665 563 (biuro akademii ul. Rydlówka 23)</t>
         </is>
       </c>
     </row>
@@ -9438,17 +9601,25 @@
           <t>Limanowa</t>
         </is>
       </c>
-      <c r="D230" s="8" t="inlineStr"/>
-      <c r="E230" s="8" t="inlineStr"/>
-      <c r="F230" s="8" t="inlineStr"/>
-      <c r="G230" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D230" s="8" t="inlineStr">
+        <is>
+          <t>Stadion im. Romana Szumilasa, ul. Józefa Marka 34, 34-600 Limanowa</t>
+        </is>
+      </c>
+      <c r="E230" s="8" t="n"/>
+      <c r="F230" s="8" t="inlineStr">
+        <is>
+          <t>https://www.limanovia.net/klub/kontakt.html</t>
+        </is>
+      </c>
+      <c r="G230" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
         </is>
       </c>
       <c r="H230" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>kierownik klubu Mateusz Wroński tel. 537 303 258; ogólnego e-maila nie znalazłem</t>
         </is>
       </c>
     </row>
@@ -9468,17 +9639,29 @@
           <t>Dębica</t>
         </is>
       </c>
-      <c r="D231" s="8" t="inlineStr"/>
-      <c r="E231" s="8" t="inlineStr"/>
-      <c r="F231" s="8" t="inlineStr"/>
-      <c r="G231" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D231" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Świętosława 89, 39-200 Dębica</t>
+        </is>
+      </c>
+      <c r="E231" s="8" t="inlineStr">
+        <is>
+          <t>biuro@dapdebica.pl</t>
+        </is>
+      </c>
+      <c r="F231" s="8" t="inlineStr">
+        <is>
+          <t>http://dapdebica.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G231" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H231" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>znaleziona tylko siedziba (adres rejestrowy) – boisko meczowe do potwierdzenia</t>
         </is>
       </c>
     </row>
@@ -9498,17 +9681,29 @@
           <t>Kielce</t>
         </is>
       </c>
-      <c r="D232" s="8" t="inlineStr"/>
-      <c r="E232" s="8" t="inlineStr"/>
-      <c r="F232" s="8" t="inlineStr"/>
-      <c r="G232" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D232" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Orląt, ul. Warszawska 338, 25-414 Kielce</t>
+        </is>
+      </c>
+      <c r="E232" s="8" t="inlineStr">
+        <is>
+          <t>info@orletakielce.pl</t>
+        </is>
+      </c>
+      <c r="F232" s="8" t="inlineStr">
+        <is>
+          <t>https://orletakielce.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G232" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H232" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>tel. 888 615 855</t>
         </is>
       </c>
     </row>
@@ -9596,17 +9791,25 @@
           <t>Kielce</t>
         </is>
       </c>
-      <c r="D235" s="8" t="inlineStr"/>
-      <c r="E235" s="8" t="inlineStr"/>
-      <c r="F235" s="8" t="inlineStr"/>
-      <c r="G235" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="D235" s="8" t="inlineStr">
+        <is>
+          <t>Exbud Arena / boisko boczne, ul. Ściegiennego 8, 25-033 Kielce</t>
+        </is>
+      </c>
+      <c r="E235" s="8" t="n"/>
+      <c r="F235" s="8" t="inlineStr">
+        <is>
+          <t>https://www.korona-kielce.pl/kontakt-akademia</t>
+        </is>
+      </c>
+      <c r="G235" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="H235" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>adres klubu i stadionu – boisko meczowe U15 do potwierdzenia; e-maile akademii zamaskowane na stronie; sekretariat tel. 41 340 34 00</t>
         </is>
       </c>
     </row>
@@ -10487,18 +10690,34 @@
           <t>Odra Opole</t>
         </is>
       </c>
-      <c r="C259" s="8" t="inlineStr"/>
-      <c r="D259" s="8" t="inlineStr"/>
-      <c r="E259" s="8" t="inlineStr"/>
-      <c r="F259" s="8" t="inlineStr"/>
-      <c r="G259" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="C259" s="8" t="inlineStr">
+        <is>
+          <t>Opole</t>
+        </is>
+      </c>
+      <c r="D259" s="8" t="inlineStr">
+        <is>
+          <t>Itaka Arena (Stadion Miejski), ul. Leonarda Olejnika 1, 45-839 Opole</t>
+        </is>
+      </c>
+      <c r="E259" s="8" t="inlineStr">
+        <is>
+          <t>klub@odraopole.pl</t>
+        </is>
+      </c>
+      <c r="F259" s="8" t="inlineStr">
+        <is>
+          <t>https://odraopole.pl/en/kontakt</t>
+        </is>
+      </c>
+      <c r="G259" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H259" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>sekretariat tel. 575 875 432; stary stadion ul. Oleska 51 już nieużywany</t>
         </is>
       </c>
     </row>
@@ -10513,18 +10732,34 @@
           <t>Bruk-Bet Termalica Nieciecza</t>
         </is>
       </c>
-      <c r="C260" s="8" t="inlineStr"/>
-      <c r="D260" s="8" t="inlineStr"/>
-      <c r="E260" s="8" t="inlineStr"/>
-      <c r="F260" s="8" t="inlineStr"/>
-      <c r="G260" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="C260" s="8" t="inlineStr">
+        <is>
+          <t>Nieciecza</t>
+        </is>
+      </c>
+      <c r="D260" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Bruk-Bet Termalica, Nieciecza 199, 33-240 Żabno</t>
+        </is>
+      </c>
+      <c r="E260" s="8" t="inlineStr">
+        <is>
+          <t>termalica@brukbet.com</t>
+        </is>
+      </c>
+      <c r="F260" s="8" t="inlineStr">
+        <is>
+          <t>https://termalica.brukbet.com/index.php/kontakt/</t>
+        </is>
+      </c>
+      <c r="G260" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H260" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>tel. 14 644 44 44; akademia: dawid.krupa@bruk-bet.pl</t>
         </is>
       </c>
     </row>
@@ -10577,18 +10812,34 @@
           <t>Puszcza Niepołomice</t>
         </is>
       </c>
-      <c r="C262" s="8" t="inlineStr"/>
-      <c r="D262" s="8" t="inlineStr"/>
-      <c r="E262" s="8" t="inlineStr"/>
-      <c r="F262" s="8" t="inlineStr"/>
-      <c r="G262" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="C262" s="8" t="inlineStr">
+        <is>
+          <t>Niepołomice</t>
+        </is>
+      </c>
+      <c r="D262" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Miejski, ul. Kusocińskiego 2, 32-005 Niepołomice</t>
+        </is>
+      </c>
+      <c r="E262" s="8" t="inlineStr">
+        <is>
+          <t>biuro@puszcza-niepolomice.pl</t>
+        </is>
+      </c>
+      <c r="F262" s="8" t="inlineStr">
+        <is>
+          <t>https://www.niepolomice.eu/informator/miejski-klub-sportowy-puszcza-niepolomice/</t>
+        </is>
+      </c>
+      <c r="G262" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H262" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>dane z informatora Gminy Niepołomice (Niepołomicki Sport S.A.); tel. 12 281 21 20</t>
         </is>
       </c>
     </row>
@@ -10633,18 +10884,34 @@
           <t>Pogoń Grodzisk Mazowiecki</t>
         </is>
       </c>
-      <c r="C264" s="8" t="inlineStr"/>
-      <c r="D264" s="8" t="inlineStr"/>
-      <c r="E264" s="8" t="inlineStr"/>
-      <c r="F264" s="8" t="inlineStr"/>
-      <c r="G264" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="C264" s="8" t="inlineStr">
+        <is>
+          <t>Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="D264" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Pogoni, al. Mokronoskich 4, 05-825 Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="E264" s="8" t="inlineStr">
+        <is>
+          <t>sekretariat@pogongrodzisk.pl</t>
+        </is>
+      </c>
+      <c r="F264" s="8" t="inlineStr">
+        <is>
+          <t>https://pogongrodzisk.pl/kontakt</t>
+        </is>
+      </c>
+      <c r="G264" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H264" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>tel. 22 120 29 07; akademia: koordynator@pogongrodzisk.pl</t>
         </is>
       </c>
     </row>
@@ -10727,18 +10994,34 @@
           <t>Pogoń Siedlce</t>
         </is>
       </c>
-      <c r="C267" s="8" t="inlineStr"/>
-      <c r="D267" s="8" t="inlineStr"/>
-      <c r="E267" s="8" t="inlineStr"/>
-      <c r="F267" s="8" t="inlineStr"/>
-      <c r="G267" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="C267" s="8" t="inlineStr">
+        <is>
+          <t>Siedlce</t>
+        </is>
+      </c>
+      <c r="D267" s="8" t="inlineStr">
+        <is>
+          <t>Stadion ARMS (ROSRRiT), ul. Jana Pawła II 6, 08-110 Siedlce</t>
+        </is>
+      </c>
+      <c r="E267" s="8" t="inlineStr">
+        <is>
+          <t>biuro@mkppogonsiedlce.pl</t>
+        </is>
+      </c>
+      <c r="F267" s="8" t="inlineStr">
+        <is>
+          <t>https://mkppogonsiedlce.pl/?page_id=94</t>
+        </is>
+      </c>
+      <c r="G267" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H267" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>biuro klubu ul. Prusa 6; tel. 25 633 36 47</t>
         </is>
       </c>
     </row>
@@ -10783,18 +11066,34 @@
           <t>Warta Poznań</t>
         </is>
       </c>
-      <c r="C269" s="8" t="inlineStr"/>
-      <c r="D269" s="8" t="inlineStr"/>
-      <c r="E269" s="8" t="inlineStr"/>
-      <c r="F269" s="8" t="inlineStr"/>
-      <c r="G269" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="C269" s="8" t="inlineStr">
+        <is>
+          <t>Poznań</t>
+        </is>
+      </c>
+      <c r="D269" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Warty „Ogródek”, ul. Droga Dębińska 12, 61-001 Poznań</t>
+        </is>
+      </c>
+      <c r="E269" s="8" t="inlineStr">
+        <is>
+          <t>info@wartapoznan.pl</t>
+        </is>
+      </c>
+      <c r="F269" s="8" t="inlineStr">
+        <is>
+          <t>https://wartapoznan.pl/</t>
+        </is>
+      </c>
+      <c r="G269" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H269" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>siedziba spółki ul. Spychalskiego 34; akademia: akademia@wartapoznan.pl</t>
         </is>
       </c>
     </row>
@@ -10843,18 +11142,34 @@
           <t>Unia Skierniewice</t>
         </is>
       </c>
-      <c r="C271" s="8" t="inlineStr"/>
-      <c r="D271" s="8" t="inlineStr"/>
-      <c r="E271" s="8" t="inlineStr"/>
-      <c r="F271" s="8" t="inlineStr"/>
-      <c r="G271" s="12" t="inlineStr">
-        <is>
-          <t>Do uzupełnienia</t>
+      <c r="C271" s="8" t="inlineStr">
+        <is>
+          <t>Skierniewice</t>
+        </is>
+      </c>
+      <c r="D271" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Miejski, ul. Pomologiczna 8, 96-100 Skierniewice</t>
+        </is>
+      </c>
+      <c r="E271" s="8" t="inlineStr">
+        <is>
+          <t>biuro@uniaskierniewice.pl</t>
+        </is>
+      </c>
+      <c r="F271" s="8" t="inlineStr">
+        <is>
+          <t>https://uniaskierniewice.pl/contact</t>
+        </is>
+      </c>
+      <c r="G271" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="H271" s="8" t="inlineStr">
         <is>
-          <t>Do uzupełnienia</t>
+          <t>e-mail biura z bilety.uniaskierniewice.pl; kierownik klubu Kamil Kaczyński tel. 667 658 195 (kamil.kaczynski@uniaskierniewice.pl z listy kontaktów)</t>
         </is>
       </c>
     </row>
@@ -10892,8 +11207,1458 @@
       </c>
       <c r="H272" s="8" t="inlineStr"/>
     </row>
+    <row r="273">
+      <c r="A273" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B273" s="8" t="inlineStr">
+        <is>
+          <t>Amator Kiełpino</t>
+        </is>
+      </c>
+      <c r="C273" s="8" t="inlineStr">
+        <is>
+          <t>Kiełpino</t>
+        </is>
+      </c>
+      <c r="D273" s="8" t="inlineStr">
+        <is>
+          <t>Stadion w Kiełpinie, ul. Długa 78A, 83-307 Kiełpino</t>
+        </is>
+      </c>
+      <c r="E273" s="8" t="inlineStr">
+        <is>
+          <t>amator.kielpino@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F273" s="8" t="inlineStr">
+        <is>
+          <t>https://www.kartuzy.pl/strona/informacje-dla-mieszkancow-obiekty-sportowe-harmonogram-korzystania/873-boisko-pilkarskie-na</t>
+        </is>
+      </c>
+      <c r="G273" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H273" s="8" t="inlineStr">
+        <is>
+          <t>adres boiska ze strony Gminy Kartuzy (obiekt w zarządzie KS Amator); e-mail z listy kontaktów (konto klubu w Pomorskim ZPN) – nie potwierdzony w źródle</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B274" s="8" t="inlineStr">
+        <is>
+          <t>Akademia Piłkarska Karol Piątek</t>
+        </is>
+      </c>
+      <c r="C274" s="8" t="inlineStr">
+        <is>
+          <t>Luzino</t>
+        </is>
+      </c>
+      <c r="D274" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Gminny w Luzinie, ul. Mickiewicza 22, 84-242 Luzino</t>
+        </is>
+      </c>
+      <c r="E274" s="8" t="inlineStr">
+        <is>
+          <t>akademia.piatek@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F274" s="8" t="inlineStr">
+        <is>
+          <t>https://lzs-pomorski.pl/klub/akademia-pilkarska-karol-piatek/</t>
+        </is>
+      </c>
+      <c r="G274" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H274" s="8" t="inlineStr">
+        <is>
+          <t>na liście kontaktów jako „Akademia Piątek”; klub działa przy GOSRiT Luzino – stadion gminny wg gosrit.luzino.pl/stadion-gminny-w-luzinie/, boisko meczowe akademii do potwierdzenia; e-mail z listy kontaktów; w Pomorskim LZS: k.piatek@gosrit.luzino.pl, tel. 501 425 426</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B275" s="8" t="inlineStr">
+        <is>
+          <t>APK Jedynka Kartuzy</t>
+        </is>
+      </c>
+      <c r="C275" s="8" t="inlineStr">
+        <is>
+          <t>Kartuzy</t>
+        </is>
+      </c>
+      <c r="D275" s="8" t="n"/>
+      <c r="E275" s="8" t="inlineStr">
+        <is>
+          <t>apkartuzy10@gmail.com</t>
+        </is>
+      </c>
+      <c r="F275" s="8" t="inlineStr">
+        <is>
+          <t>https://apkjedynka.pl/</t>
+        </is>
+      </c>
+      <c r="G275" s="9" t="inlineStr">
+        <is>
+          <t>Do uzupełnienia</t>
+        </is>
+      </c>
+      <c r="H275" s="8" t="inlineStr">
+        <is>
+          <t>Akademia Piłkarska Kartuzy (KRS 752774), na liście kontaktów jako „AP Kartuzy”; e-mail ze strony klubu; adresu boiska strona nie podaje (treningi na obiektach w Kartuzach); tel. 793 091 111</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B276" s="8" t="inlineStr">
+        <is>
+          <t>AS Piłeczka Pruszcz Gdański</t>
+        </is>
+      </c>
+      <c r="C276" s="8" t="inlineStr">
+        <is>
+          <t>Pruszcz Gdański</t>
+        </is>
+      </c>
+      <c r="D276" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Jacka Soplicy 10/12, 83-000 Pruszcz Gdański</t>
+        </is>
+      </c>
+      <c r="E276" s="8" t="inlineStr">
+        <is>
+          <t>as.pileczka@tlen.pl</t>
+        </is>
+      </c>
+      <c r="F276" s="8" t="inlineStr">
+        <is>
+          <t>https://aspileczka.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G276" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H276" s="8" t="inlineStr">
+        <is>
+          <t>Akademia Sportu Piłeczka; znaleziona tylko siedziba – obiekty treningowe klub podaje po zapisie; na stronie e-mail @tlen.pl, na liście kontaktów as.pileczka@o2.pl – sprawdź, który aktualny; tel. 504 189 453</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B277" s="8" t="inlineStr">
+        <is>
+          <t>Brda Przechlewo</t>
+        </is>
+      </c>
+      <c r="C277" s="8" t="inlineStr">
+        <is>
+          <t>Przechlewo</t>
+        </is>
+      </c>
+      <c r="D277" s="8" t="inlineStr">
+        <is>
+          <t>Stadion OSiR, ul. Szkolna 23, 77-320 Przechlewo</t>
+        </is>
+      </c>
+      <c r="E277" s="8" t="inlineStr">
+        <is>
+          <t>brda.przechlewo@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F277" s="8" t="inlineStr">
+        <is>
+          <t>https://www.osir.przechlewo.pl/stadiony-pilkarskie.html</t>
+        </is>
+      </c>
+      <c r="G277" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H277" s="8" t="inlineStr">
+        <is>
+          <t>stadion gminnego OSiR Przechlewo – że Brda gra tam mecze, nie potwierdziłem w źródle klubu/związku; e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B278" s="8" t="inlineStr">
+        <is>
+          <t>Broń Radom</t>
+        </is>
+      </c>
+      <c r="C278" s="8" t="inlineStr">
+        <is>
+          <t>Radom</t>
+        </is>
+      </c>
+      <c r="D278" s="8" t="inlineStr">
+        <is>
+          <t>Stadion MOSiR, ul. Narutowicza 9, 26-600 Radom</t>
+        </is>
+      </c>
+      <c r="E278" s="8" t="inlineStr">
+        <is>
+          <t>klub@bronradom.pl</t>
+        </is>
+      </c>
+      <c r="F278" s="8" t="inlineStr">
+        <is>
+          <t>https://bronradom.pl/informacje-o-klubie/</t>
+        </is>
+      </c>
+      <c r="G278" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H278" s="8" t="inlineStr">
+        <is>
+          <t>siedziba pod trybuną A; tel. 721 866 320</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B279" s="8" t="inlineStr">
+        <is>
+          <t>Bałtyk Sztutowo</t>
+        </is>
+      </c>
+      <c r="C279" s="8" t="inlineStr">
+        <is>
+          <t>Sztutowo</t>
+        </is>
+      </c>
+      <c r="D279" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Gminny, ul. Obozowa 16, 82-110 Sztutowo</t>
+        </is>
+      </c>
+      <c r="E279" s="8" t="inlineStr">
+        <is>
+          <t>baltyk.sztutowo@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F279" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sztutowo.pl/zajecia-gimnastyczne-dla-seniorow/</t>
+        </is>
+      </c>
+      <c r="G279" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H279" s="8" t="inlineStr">
+        <is>
+          <t>adres stadionu gminnego ze strony Urzędu Gminy Sztutowo; e-mail z listy kontaktów (konto klubu w Pomorskim ZPN) – nie potwierdzony w źródle</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B280" s="8" t="inlineStr">
+        <is>
+          <t>Czarni Przemysław</t>
+        </is>
+      </c>
+      <c r="C280" s="8" t="inlineStr">
+        <is>
+          <t>Przemysław</t>
+        </is>
+      </c>
+      <c r="D280" s="8" t="inlineStr">
+        <is>
+          <t>SportPlac, Przemysław 1, 82-103 Stegna</t>
+        </is>
+      </c>
+      <c r="E280" s="8" t="inlineStr">
+        <is>
+          <t>czarni.przemyslaw@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F280" s="8" t="inlineStr">
+        <is>
+          <t>https://www.laczynaspilka.pl/rozgrywki/mecz/ks-mady-ostaszewo,st-drewnica-czarni-przemyslaw,2306657.html</t>
+        </is>
+      </c>
+      <c r="G280" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H280" s="8" t="inlineStr">
+        <is>
+          <t>obiekt z terminarza Łączy Nas Piłka; kod pocztowy wg adresu klubu (Przemysław 52, 82-103 Stegna); e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B281" s="8" t="inlineStr">
+        <is>
+          <t>GKS Wikielec</t>
+        </is>
+      </c>
+      <c r="C281" s="8" t="inlineStr">
+        <is>
+          <t>Wikielec</t>
+        </is>
+      </c>
+      <c r="D281" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Gminny w Wikielcu, ul. Bukowa 80, 14-200 Iława</t>
+        </is>
+      </c>
+      <c r="E281" s="8" t="inlineStr">
+        <is>
+          <t>gkswikielec@wmzpn.pl</t>
+        </is>
+      </c>
+      <c r="F281" s="8" t="inlineStr">
+        <is>
+          <t>https://gkswikielec.pl/kontakt</t>
+        </is>
+      </c>
+      <c r="G281" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H281" s="8" t="inlineStr">
+        <is>
+          <t>dawny adres Wikielec 65B (zmiana po nadaniu nazw ulic); tel. 509 424 466</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B282" s="8" t="inlineStr">
+        <is>
+          <t>Iskra Malbork</t>
+        </is>
+      </c>
+      <c r="C282" s="8" t="inlineStr">
+        <is>
+          <t>Malbork</t>
+        </is>
+      </c>
+      <c r="D282" s="8" t="n"/>
+      <c r="E282" s="8" t="inlineStr">
+        <is>
+          <t>iskra.malbork@gmail.com</t>
+        </is>
+      </c>
+      <c r="F282" s="8" t="n"/>
+      <c r="G282" s="9" t="inlineStr">
+        <is>
+          <t>Do uzupełnienia</t>
+        </is>
+      </c>
+      <c r="H282" s="8" t="inlineStr">
+        <is>
+          <t>prawdopodobnie Gminna Akademia Sportowa Iskra Malbork (KRS 0000933634, siedziba rejestrowa Lasowice Wielkie 65A, 82-200 Malbork) – boiska nie znalazłem na stronie klubu/związku/gminy; e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B283" s="8" t="inlineStr">
+        <is>
+          <t>Chełminianka Chełmno</t>
+        </is>
+      </c>
+      <c r="C283" s="8" t="inlineStr">
+        <is>
+          <t>Chełmno</t>
+        </is>
+      </c>
+      <c r="D283" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Polna 11, 86-200 Chełmno</t>
+        </is>
+      </c>
+      <c r="E283" s="8" t="inlineStr">
+        <is>
+          <t>chelminiankachelmno@gazeta.pl</t>
+        </is>
+      </c>
+      <c r="F283" s="8" t="inlineStr">
+        <is>
+          <t>https://chelmno.pl/organizacje-pozarzadowe/</t>
+        </is>
+      </c>
+      <c r="G283" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H283" s="8" t="inlineStr">
+        <is>
+          <t>dane z wykazu organizacji na stronie Miasta Chełmno – możliwe, że to biuro, nie boisko; tel. 506 822 675; UWAGA: e-mail z listy kontaktów sekretariat@chelmianka.pl to domena Chełmianki Chełm (inny klub, jest w bazie) – sprawdź, o który klub chodzi</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B284" s="8" t="inlineStr">
+        <is>
+          <t>KS Pszczółki</t>
+        </is>
+      </c>
+      <c r="C284" s="8" t="inlineStr">
+        <is>
+          <t>Pszczółki</t>
+        </is>
+      </c>
+      <c r="D284" s="8" t="inlineStr">
+        <is>
+          <t>Stadion im. 700-lecia Pszczółek, ul. Sportowa 27, 83-032 Pszczółki</t>
+        </is>
+      </c>
+      <c r="E284" s="8" t="inlineStr">
+        <is>
+          <t>ks.pszczolki@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F284" s="8" t="inlineStr">
+        <is>
+          <t>https://pszczolki.pl/obiekty-sportowe.html</t>
+        </is>
+      </c>
+      <c r="G284" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H284" s="8" t="inlineStr">
+        <is>
+          <t>stadion gminny ze strony Gminy Pszczółki (strona nie wymienia klubu wprost); e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B285" s="8" t="inlineStr">
+        <is>
+          <t>UKS Skarszewy</t>
+        </is>
+      </c>
+      <c r="C285" s="8" t="inlineStr">
+        <is>
+          <t>Skarszewy</t>
+        </is>
+      </c>
+      <c r="D285" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Miejski, ul. Wybickiego 10, 83-250 Skarszewy</t>
+        </is>
+      </c>
+      <c r="E285" s="8" t="inlineStr">
+        <is>
+          <t>biuro@uksskarszewy.pl</t>
+        </is>
+      </c>
+      <c r="F285" s="8" t="inlineStr">
+        <is>
+          <t>http://uksskarszewy.pl/contact</t>
+        </is>
+      </c>
+      <c r="G285" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H285" s="8" t="inlineStr">
+        <is>
+          <t>na liście kontaktów jako „KS Skarszewy”; e-mail ze strony klubu; adres stadionu miejskiego (GOSiR) ze strony Gminy Skarszewy – że UKS gra tam mecze, nie potwierdziłem; tel. 691 844 123</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B286" s="8" t="inlineStr">
+        <is>
+          <t>Skra Częstochowa</t>
+        </is>
+      </c>
+      <c r="C286" s="8" t="inlineStr">
+        <is>
+          <t>Częstochowa</t>
+        </is>
+      </c>
+      <c r="D286" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Skry, ul. Loretańska 20, 42-200 Częstochowa</t>
+        </is>
+      </c>
+      <c r="E286" s="8" t="inlineStr">
+        <is>
+          <t>sekretariat@ks-skra.pl</t>
+        </is>
+      </c>
+      <c r="F286" s="8" t="inlineStr">
+        <is>
+          <t>https://ks-skra.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G286" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H286" s="8" t="inlineStr">
+        <is>
+          <t>sekretariat: aleksandra.kmiec@ks-skra.pl, tel. 608 21 41 91</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B287" s="8" t="inlineStr">
+        <is>
+          <t>KS Wasilków</t>
+        </is>
+      </c>
+      <c r="C287" s="8" t="inlineStr">
+        <is>
+          <t>Wasilków</t>
+        </is>
+      </c>
+      <c r="D287" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Miejski, ul. Supraślska 21, 16-010 Wasilków</t>
+        </is>
+      </c>
+      <c r="E287" s="8" t="inlineStr">
+        <is>
+          <t>poczta@kswasilkow.pl</t>
+        </is>
+      </c>
+      <c r="F287" s="8" t="inlineStr">
+        <is>
+          <t>https://kswasilkow.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G287" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H287" s="8" t="inlineStr">
+        <is>
+          <t>biuro: ul. Białostocka 7; tel. 85 718 52 03; akademia tel. 512 570 511</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B288" s="8" t="inlineStr">
+        <is>
+          <t>Noteć Gębice</t>
+        </is>
+      </c>
+      <c r="C288" s="8" t="inlineStr">
+        <is>
+          <t>Gębice</t>
+        </is>
+      </c>
+      <c r="D288" s="8" t="inlineStr">
+        <is>
+          <t>Boisko w Gębicach, ul. Wolności, 88-330 Gębice</t>
+        </is>
+      </c>
+      <c r="E288" s="8" t="n"/>
+      <c r="F288" s="8" t="inlineStr">
+        <is>
+          <t>https://mogilnosport.pl/obiekty/obiekty-sportowe-i-rekreacyjne/gebice/</t>
+        </is>
+      </c>
+      <c r="G288" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H288" s="8" t="inlineStr">
+        <is>
+          <t>pełnowymiarowe boisko trawiaste przy ul. Wolności (obiekty sportowe gminy Mogilno), po południu korzystają sekcje klubu; numer posesji i kod pocztowy do potwierdzenia; e-maila nie znalazłem</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B289" s="8" t="inlineStr">
+        <is>
+          <t>Ogniwo Sopot</t>
+        </is>
+      </c>
+      <c r="C289" s="8" t="inlineStr">
+        <is>
+          <t>Sopot</t>
+        </is>
+      </c>
+      <c r="D289" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Miejski im. Edwarda Hodury, ul. Jana z Kolna 18, 81-741 Sopot</t>
+        </is>
+      </c>
+      <c r="E289" s="8" t="inlineStr">
+        <is>
+          <t>ogniwo@ogniwosopot.pl</t>
+        </is>
+      </c>
+      <c r="F289" s="8" t="inlineStr">
+        <is>
+          <t>https://ogniwosopot.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G289" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H289" s="8" t="inlineStr">
+        <is>
+          <t>dyrektor klubu tel. 795 944 441; koordynator grup U15: k.szymanski@ogniwosopot.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B290" s="8" t="inlineStr">
+        <is>
+          <t>UKS Orły Tczew</t>
+        </is>
+      </c>
+      <c r="C290" s="8" t="inlineStr">
+        <is>
+          <t>Tczew</t>
+        </is>
+      </c>
+      <c r="D290" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Podmurna 11, 83-110 Tczew</t>
+        </is>
+      </c>
+      <c r="E290" s="8" t="inlineStr">
+        <is>
+          <t>klub@orlytczew.pl</t>
+        </is>
+      </c>
+      <c r="F290" s="8" t="inlineStr">
+        <is>
+          <t>http://orlytczew.pl/</t>
+        </is>
+      </c>
+      <c r="G290" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H290" s="8" t="inlineStr">
+        <is>
+          <t>dane ze strony klubu (wpisy do 2016 r.); mecze grane na stadionie przy ul. Bałdowskiej – numer i aktualność do potwierdzenia; na liście kontaktów gwolski@orlytczew.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B291" s="8" t="inlineStr">
+        <is>
+          <t>Pogoń Prabuty</t>
+        </is>
+      </c>
+      <c r="C291" s="8" t="inlineStr">
+        <is>
+          <t>Prabuty</t>
+        </is>
+      </c>
+      <c r="D291" s="8" t="inlineStr">
+        <is>
+          <t>Stadion MKS Pogoń, ul. Jagiełły, 82-550 Prabuty</t>
+        </is>
+      </c>
+      <c r="E291" s="8" t="inlineStr">
+        <is>
+          <t>pogon.prabuty@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F291" s="8" t="inlineStr">
+        <is>
+          <t>https://www.prabuty.pl/stadion-mks-pogon/</t>
+        </is>
+      </c>
+      <c r="G291" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H291" s="8" t="inlineStr">
+        <is>
+          <t>ze strony Gminy Prabuty: na stadionie trenują i grają mecze ligowe seniorzy i juniorzy klubu; obiekt prowadzi Prabuckie Centrum Kultury i Sportu; numer posesji do potwierdzenia; e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B292" s="8" t="inlineStr">
+        <is>
+          <t>Pokolenia Lechii Gdańsk</t>
+        </is>
+      </c>
+      <c r="C292" s="8" t="inlineStr">
+        <is>
+          <t>Gdańsk</t>
+        </is>
+      </c>
+      <c r="D292" s="8" t="inlineStr">
+        <is>
+          <t>ul. Zielonogórska 4, Gdańsk</t>
+        </is>
+      </c>
+      <c r="E292" s="8" t="inlineStr">
+        <is>
+          <t>pokolenia.lechii.gda@wp.pl</t>
+        </is>
+      </c>
+      <c r="F292" s="8" t="inlineStr">
+        <is>
+          <t>https://www.gdansk.pl/urzad-miejski/biuro-prezydenta-ds-sportu/gdanskie-kluby-zapraszaja-dzieci-i-mlodziez,a,43554</t>
+        </is>
+      </c>
+      <c r="G292" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H292" s="8" t="inlineStr">
+        <is>
+          <t>szkółka piłkarska (nie Akademia Lechii); adres z listy klubów na stronie Miasta Gdańsk (ok. 2015) – nowsze katalogi podają ul. Traugutta 29, 80-034 Gdańsk; kod pocztowy i boisko do potwierdzenia; e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B293" s="8" t="inlineStr">
+        <is>
+          <t>Sławek Borzechowo</t>
+        </is>
+      </c>
+      <c r="C293" s="8" t="inlineStr">
+        <is>
+          <t>Borzechowo</t>
+        </is>
+      </c>
+      <c r="D293" s="8" t="inlineStr">
+        <is>
+          <t>Boisko sportowe, ul. Szkolna 3, 83-224 Borzechowo</t>
+        </is>
+      </c>
+      <c r="E293" s="8" t="inlineStr">
+        <is>
+          <t>slawekborzechowo1@gmail.com</t>
+        </is>
+      </c>
+      <c r="F293" s="8" t="inlineStr">
+        <is>
+          <t>http://slawekborzechowo.5v.pl/</t>
+        </is>
+      </c>
+      <c r="G293" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H293" s="8" t="inlineStr">
+        <is>
+          <t>e-mail ze strony klubu, adres ul. Szkolna 3 z profilu klubu na FB – czy to boisko, do potwierdzenia; na liście kontaktów slawek.borzechowo@pomorski-zpn.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B294" s="8" t="inlineStr">
+        <is>
+          <t>Sokół Zblewo</t>
+        </is>
+      </c>
+      <c r="C294" s="8" t="inlineStr">
+        <is>
+          <t>Zblewo</t>
+        </is>
+      </c>
+      <c r="D294" s="8" t="inlineStr">
+        <is>
+          <t>Stadion w Zblewie, ul. Sportowa 7, 83-210 Zblewo</t>
+        </is>
+      </c>
+      <c r="E294" s="8" t="inlineStr">
+        <is>
+          <t>sokol.zblewo@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F294" s="8" t="inlineStr">
+        <is>
+          <t>https://powiatstarogard.pl/organizacje/klub-sportowy-sokol-zblewo/</t>
+        </is>
+      </c>
+      <c r="G294" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H294" s="8" t="inlineStr">
+        <is>
+          <t>adres klubu z wykazu organizacji Powiatu Starogardzkiego (inne katalogi: Sportowa 27); stadion gminny przy ul. Sportowej – numer do potwierdzenia; e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B295" s="8" t="inlineStr">
+        <is>
+          <t>Stomil Olsztyn</t>
+        </is>
+      </c>
+      <c r="C295" s="8" t="inlineStr">
+        <is>
+          <t>Olsztyn</t>
+        </is>
+      </c>
+      <c r="D295" s="8" t="inlineStr">
+        <is>
+          <t>Stadion OSiR, al. Piłsudskiego 69a, 10-449 Olsztyn</t>
+        </is>
+      </c>
+      <c r="E295" s="8" t="inlineStr">
+        <is>
+          <t>biuro@stomilolsztyn.com</t>
+        </is>
+      </c>
+      <c r="F295" s="8" t="inlineStr">
+        <is>
+          <t>https://www.stomilolsztyn.com/kontakt/</t>
+        </is>
+      </c>
+      <c r="G295" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H295" s="8" t="inlineStr">
+        <is>
+          <t>tel. 89 534 12 38; akademia: stomilolsztyn.com/kontakt-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B296" s="8" t="inlineStr">
+        <is>
+          <t>Supra Kwidzyn</t>
+        </is>
+      </c>
+      <c r="C296" s="8" t="inlineStr">
+        <is>
+          <t>Kwidzyn</t>
+        </is>
+      </c>
+      <c r="D296" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Sportowa 6, 82-500 Kwidzyn</t>
+        </is>
+      </c>
+      <c r="E296" s="8" t="inlineStr">
+        <is>
+          <t>supra.kwidzyn@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F296" s="8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100063858990742</t>
+        </is>
+      </c>
+      <c r="G296" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H296" s="8" t="inlineStr">
+        <is>
+          <t>Stowarzyszenie Rozwoju Sportu Supra; adres z profilu klubu na FB (ten sam w KRS) – czy to boisko meczowe, do potwierdzenia; e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B297" s="8" t="inlineStr">
+        <is>
+          <t>Świdniczanka Świdnik</t>
+        </is>
+      </c>
+      <c r="C297" s="8" t="inlineStr">
+        <is>
+          <t>Świdnik</t>
+        </is>
+      </c>
+      <c r="D297" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Kosynierów 17B, 21-040 Świdnik</t>
+        </is>
+      </c>
+      <c r="E297" s="8" t="inlineStr">
+        <is>
+          <t>kontakt@ksswidniczanka.pl</t>
+        </is>
+      </c>
+      <c r="F297" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ksswidniczanka.pl/kontakt.html</t>
+        </is>
+      </c>
+      <c r="G297" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H297" s="8" t="inlineStr">
+        <is>
+          <t>znaleziona tylko siedziba; obiekt meczowy (dawniej boisko przy ul. Turystycznej) do potwierdzenia w terminarzu; tel. 570 716 873</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B298" s="8" t="inlineStr">
+        <is>
+          <t>Stal Kraśnik</t>
+        </is>
+      </c>
+      <c r="C298" s="8" t="inlineStr">
+        <is>
+          <t>Kraśnik</t>
+        </is>
+      </c>
+      <c r="D298" s="8" t="inlineStr">
+        <is>
+          <t>Stadion MOSiR, ul. Żwirki i Wigury 2, 23-204 Kraśnik</t>
+        </is>
+      </c>
+      <c r="E298" s="8" t="inlineStr">
+        <is>
+          <t>fksstal@krasnik.info</t>
+        </is>
+      </c>
+      <c r="F298" s="8" t="inlineStr">
+        <is>
+          <t>https://www.stalkrasnik.com/</t>
+        </is>
+      </c>
+      <c r="G298" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H298" s="8" t="inlineStr">
+        <is>
+          <t>FKS Stal; siedziba al. Niepodległości 44, 23-210 Kraśnik (krasnik.eu); stadion MOSiR wg stalkrasnik.com; e-mail z listy kontaktów (domena dawnej strony stal.krasnik.info) – portal miasta podaje kontakt czelejmagda@gmail.com, tel. 601 988 984</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B299" s="8" t="inlineStr">
+        <is>
+          <t>Tłuchovia Tłuchowo</t>
+        </is>
+      </c>
+      <c r="C299" s="8" t="inlineStr">
+        <is>
+          <t>Tłuchowo</t>
+        </is>
+      </c>
+      <c r="D299" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Gminny, ul. Sportowa 3, 87-605 Tłuchowo</t>
+        </is>
+      </c>
+      <c r="E299" s="8" t="inlineStr">
+        <is>
+          <t>d.mocki@tluchovia.pl</t>
+        </is>
+      </c>
+      <c r="F299" s="8" t="inlineStr">
+        <is>
+          <t>https://tluchovia.pl/index.php/contact-page/</t>
+        </is>
+      </c>
+      <c r="G299" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H299" s="8" t="inlineStr">
+        <is>
+          <t>GZS Tłuchovia; adres i stadion gminny ze strony klubu (nr posesji stadionu nie jest podany osobno); ogólnego e-maila brak – na stronie e-maile działaczy (m.in. d.mocki@, s.kucinski@tluchovia.pl); tel. 691 416 904</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B300" s="8" t="inlineStr">
+        <is>
+          <t>TOP 54 Biała Podlaska</t>
+        </is>
+      </c>
+      <c r="C300" s="8" t="inlineStr">
+        <is>
+          <t>Biała Podlaska</t>
+        </is>
+      </c>
+      <c r="D300" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Piłsudskiego 38, 21-500 Biała Podlaska</t>
+        </is>
+      </c>
+      <c r="E300" s="8" t="inlineStr">
+        <is>
+          <t>appodlasie@gmail.com</t>
+        </is>
+      </c>
+      <c r="F300" s="8" t="inlineStr">
+        <is>
+          <t>https://mkspodlasie1957.pl/kontakt</t>
+        </is>
+      </c>
+      <c r="G300" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H300" s="8" t="inlineStr">
+        <is>
+          <t>Akademia Piłkarska TOP 54 działa obecnie przy MKS Podlasie (strona mkspodlasie1957.pl); boiska akademii przy ul. Zdanowskiego – numer do potwierdzenia; na liście kontaktów stary e-mail aptop54@o2.pl; biuro tel. 83 343 22 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B301" s="8" t="inlineStr">
+        <is>
+          <t>Unia Klawkowo</t>
+        </is>
+      </c>
+      <c r="C301" s="8" t="inlineStr">
+        <is>
+          <t>Klawkowo</t>
+        </is>
+      </c>
+      <c r="D301" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Dębowa 3, Klawkowo, 89-620 Chojnice</t>
+        </is>
+      </c>
+      <c r="E301" s="8" t="inlineStr">
+        <is>
+          <t>unia.klawkowo@pomorski-zpn.pl</t>
+        </is>
+      </c>
+      <c r="F301" s="8" t="inlineStr">
+        <is>
+          <t>https://www.powiat.chojnice.pl/asp/pliki/aktualnosci_2021/baza_danych_organizacji_pozarzadowych_powiat_chojnicki_05.07.pdf</t>
+        </is>
+      </c>
+      <c r="G301" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H301" s="8" t="inlineStr">
+        <is>
+          <t>Wiejski Klub Sportowy; adres z bazy NGO Powiatu Chojnickiego (2021) – klub gra na własnym boisku w Klawkowie, adres boiska do potwierdzenia; e-mail z listy kontaktów</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B302" s="8" t="inlineStr">
+        <is>
+          <t>Unia Solec Kujawski</t>
+        </is>
+      </c>
+      <c r="C302" s="8" t="inlineStr">
+        <is>
+          <t>Solec Kujawski</t>
+        </is>
+      </c>
+      <c r="D302" s="8" t="inlineStr">
+        <is>
+          <t>Stadion OSiR, ul. Sportowa 1, 86-050 Solec Kujawski</t>
+        </is>
+      </c>
+      <c r="E302" s="8" t="inlineStr">
+        <is>
+          <t>ksunia.soleckujawski@o2.pl</t>
+        </is>
+      </c>
+      <c r="F302" s="8" t="inlineStr">
+        <is>
+          <t>https://uniasoleckuj.futbolowo.pl/kontakt</t>
+        </is>
+      </c>
+      <c r="G302" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H302" s="8" t="inlineStr">
+        <is>
+          <t>adres klubu = stadion OSiR; strona kontaktowa klubu sprzed ok. 4 lat – e-mail warto potwierdzić; obiekt prowadzi OSiR Solec Kujawski</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B303" s="8" t="inlineStr">
+        <is>
+          <t>Znicz Biała Piska</t>
+        </is>
+      </c>
+      <c r="C303" s="8" t="inlineStr">
+        <is>
+          <t>Biała Piska</t>
+        </is>
+      </c>
+      <c r="D303" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Miejski, ul. Sportowa 1, 12-230 Biała Piska</t>
+        </is>
+      </c>
+      <c r="E303" s="8" t="inlineStr">
+        <is>
+          <t>zniczbialapiska@wmzpn.pl</t>
+        </is>
+      </c>
+      <c r="F303" s="8" t="inlineStr">
+        <is>
+          <t>https://zniczbialapiska.pl/stadion/</t>
+        </is>
+      </c>
+      <c r="G303" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H303" s="8" t="inlineStr">
+        <is>
+          <t>biuro: Plac Mickiewicza 25; tel. 87 424 13 51</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B304" s="8" t="inlineStr">
+        <is>
+          <t>MUKS Żaki Szczecin</t>
+        </is>
+      </c>
+      <c r="C304" s="8" t="inlineStr">
+        <is>
+          <t>Szczecin</t>
+        </is>
+      </c>
+      <c r="D304" s="8" t="inlineStr">
+        <is>
+          <t>siedziba: ul. Pomorska 150, 70-812 Szczecin</t>
+        </is>
+      </c>
+      <c r="E304" s="8" t="inlineStr">
+        <is>
+          <t>muks@zaki.szczecin.pl</t>
+        </is>
+      </c>
+      <c r="F304" s="8" t="inlineStr">
+        <is>
+          <t>https://mukszaki.pl/kontakt</t>
+        </is>
+      </c>
+      <c r="G304" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H304" s="8" t="inlineStr">
+        <is>
+          <t>znaleziona tylko siedziba – boisko meczowe do potwierdzenia; na liście kontaktów mukszaki@gmail.com; osobne stowarzyszenie Akademia Piłkarska Żaki: ul. Portowa 21, akademia@zaki.szczecin.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B305" s="8" t="inlineStr">
+        <is>
+          <t>Wisła Puławy</t>
+        </is>
+      </c>
+      <c r="C305" s="8" t="inlineStr">
+        <is>
+          <t>Puławy</t>
+        </is>
+      </c>
+      <c r="D305" s="8" t="inlineStr">
+        <is>
+          <t>Stadion MOSiR, ul. Hauke-Bosaka 1, 24-100 Puławy</t>
+        </is>
+      </c>
+      <c r="E305" s="8" t="inlineStr">
+        <is>
+          <t>sekretariat@kswislapulawy.pl</t>
+        </is>
+      </c>
+      <c r="F305" s="8" t="inlineStr">
+        <is>
+          <t>https://mosir.pulawy.pl/</t>
+        </is>
+      </c>
+      <c r="G305" s="9" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="H305" s="8" t="inlineStr">
+        <is>
+          <t>adres klubu i stadionu wg kswislapulawy.pl; mecze Wisły na stadionie potwierdzone w zapowiedziach MOSiR Puławy (2026, klasa A); tel. 81 470 49 09</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B306" s="8" t="inlineStr">
+        <is>
+          <t>Kaszubia Kościerzyna</t>
+        </is>
+      </c>
+      <c r="C306" s="8" t="inlineStr">
+        <is>
+          <t>Kościerzyna</t>
+        </is>
+      </c>
+      <c r="D306" s="8" t="inlineStr">
+        <is>
+          <t>ul. Kamienna 7, 83-400 Kościerzyna</t>
+        </is>
+      </c>
+      <c r="E306" s="8" t="inlineStr">
+        <is>
+          <t>sekretariat@kskaszubia.pl</t>
+        </is>
+      </c>
+      <c r="F306" s="8" t="inlineStr">
+        <is>
+          <t>https://akademia.kskaszubia.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="G306" s="11" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="H306" s="8" t="inlineStr">
+        <is>
+          <t>na liście kontaktów jako „AP Kaszubia Kościerzyna” (ap.koscierzyna@pomorski-zpn.pl, akademia@kskaszubia.pl); adres kontaktowy klubu – czy to stadion, do potwierdzenia; akademia tel. 733 302 000</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="8" t="inlineStr">
+        <is>
+          <t>Kontakty (spoza bazy)</t>
+        </is>
+      </c>
+      <c r="B307" s="8" t="inlineStr">
+        <is>
+          <t>Start Pruszcz</t>
+        </is>
+      </c>
+      <c r="C307" s="8" t="inlineStr">
+        <is>
+          <t>Pruszcz</t>
+        </is>
+      </c>
+      <c r="D307" s="8" t="inlineStr">
+        <is>
+          <t>Stadion Gminny, ul. Sportowa, 86-120 Pruszcz</t>
+        </is>
+      </c>
+      <c r="E307" s="8" t="n"/>
+      <c r="F307" s="8" t="inlineStr">
+        <is>
+          <t>https://pruszcz.pl/strona/216-kluby-sportowe</t>
+        </is>
+      </c>
+      <c r="G307" s="10" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+      <c r="H307" s="8" t="inlineStr">
+        <is>
+          <t>LKS Start; ze strony Gminy Pruszcz: adres klubu ul. Sportowa 8, stadion przy ul. Sportowej prowadzi GOKSiR (ul. Sportowa 10A) – numer posesji boiska do potwierdzenia; e-maila nie znalazłem</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H272"/>
+  <autoFilter ref="A1:H307"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>